<commit_message>
feat: adicionado backup e exportacao de dados
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sette-log-importacao-template.xlsx
+++ b/frontend/public/templates/sette-log-importacao-template.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="instrucoes" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="regras-importacao" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="regras-importação" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="veiculos" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="motoristas" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="abastecimentos" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="manutencoes" state="visible" r:id="rId9"/>
+    <sheet sheetId="6" name="manutenções" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="documentos" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -19,25 +19,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="176">
   <si>
-    <t>Template de importacao Sette Log</t>
+    <t>Template de importação Sette Log</t>
   </si>
   <si>
     <t>Ordem correta</t>
   </si>
   <si>
-    <t>1 veiculos, 2 motoristas, 3 abastecimentos, 4 manutencoes, 5 documentos.</t>
-  </si>
-  <si>
-    <t>Abas importaveis</t>
-  </si>
-  <si>
-    <t>Preencha apenas veiculos, motoristas, abastecimentos, manutencoes e documentos.</t>
-  </si>
-  <si>
-    <t>Cabecalho</t>
-  </si>
-  <si>
-    <t>Nao altere a primeira linha das abas importaveis.</t>
+    <t>1 veículos, 2 motoristas, 3 abastecimentos, 4 manutenções, 5 documentos.</t>
+  </si>
+  <si>
+    <t>Abas importáveis</t>
+  </si>
+  <si>
+    <t>Preencha apenas veículos, motoristas, abastecimentos, manutenções e documentos.</t>
+  </si>
+  <si>
+    <t>Cabeçalho</t>
+  </si>
+  <si>
+    <t>Não altere a primeira linha das abas importáveis.</t>
   </si>
   <si>
     <t>Exemplos</t>
@@ -58,10 +58,10 @@
     <t>Use numeros sem simbolo de moeda. Ex: 434 ou 434,50.</t>
   </si>
   <si>
-    <t>Recalculo de combustivel</t>
-  </si>
-  <si>
-    <t>Na tela de importacao, marque a opcao de recalcular valor_total quando quiser usar litros x preco_litro.</t>
+    <t>Recalculo de combustível</t>
+  </si>
+  <si>
+    <t>Na tela de importação, marque a opcao de recalcular valor_total quando quiser usar litros x preco_litro.</t>
   </si>
   <si>
     <t>Regras e campos aceitos</t>
@@ -82,19 +82,19 @@
     <t>placa *</t>
   </si>
   <si>
-    <t>Obrigatorio. Placa unica do veiculo.</t>
+    <t>Obrigatorio. Placa única do veículo.</t>
   </si>
   <si>
     <t>marca *</t>
   </si>
   <si>
-    <t>Obrigatorio. Fabricante do veiculo.</t>
+    <t>Obrigatorio. Fabricante do veículo.</t>
   </si>
   <si>
     <t>modelo *</t>
   </si>
   <si>
-    <t>Obrigatorio. Modelo do veiculo.</t>
+    <t>Obrigatorio. Modelo do veículo.</t>
   </si>
   <si>
     <t>apelido</t>
@@ -106,7 +106,7 @@
     <t>ano</t>
   </si>
   <si>
-    <t>Opcional. Ano do veiculo.</t>
+    <t>Opcional. Ano do veículo.</t>
   </si>
   <si>
     <t>tipo</t>
@@ -154,19 +154,19 @@
     <t>cidade</t>
   </si>
   <si>
-    <t>Opcional. Cidade de operacao.</t>
+    <t>Opcional. Cidade de operação.</t>
   </si>
   <si>
     <t>regra</t>
   </si>
   <si>
-    <t>A placa e a chave unica. Se ja existir, o veiculo sera atualizado.</t>
-  </si>
-  <si>
-    <t>Linhas sem placa nao sao importadas.</t>
-  </si>
-  <si>
-    <t>Veiculo inativo ou bloqueado nao deve ser usado como disponivel na operacao.</t>
+    <t>A placa e a chave única. Se já existir, o veículo será atualizado.</t>
+  </si>
+  <si>
+    <t>Linhas sem placa não sao importadas.</t>
+  </si>
+  <si>
+    <t>Veículo inativo ou bloqueado não deve ser usado como disponível na operação.</t>
   </si>
   <si>
     <t>motoristas</t>
@@ -181,7 +181,7 @@
     <t>cnh *</t>
   </si>
   <si>
-    <t>Obrigatorio. CNH unica do motorista.</t>
+    <t>Obrigatorio. CNH única do motorista.</t>
   </si>
   <si>
     <t>categoria_cnh *</t>
@@ -217,19 +217,19 @@
     <t>Opcional. active, inactive, blocked, vacation.</t>
   </si>
   <si>
-    <t>A CNH e a chave unica. Se ja existir, o motorista sera atualizado.</t>
+    <t>A CNH e a chave única. Se já existir, o motorista será atualizado.</t>
   </si>
   <si>
     <t>CNHs duplicadas dentro da mesma planilha sao bloqueadas.</t>
   </si>
   <si>
-    <t>Linhas sem nome ou sem CNH nao sao importadas.</t>
+    <t>Linhas sem nome ou sem CNH não sao importadas.</t>
   </si>
   <si>
     <t>abastecimentos</t>
   </si>
   <si>
-    <t>Obrigatorio. Placa de veiculo ja cadastrado.</t>
+    <t>Obrigatorio. Placa de veículo já cadastrado.</t>
   </si>
   <si>
     <t>litros *</t>
@@ -271,13 +271,13 @@
     <t>Opcional. Local do abastecimento.</t>
   </si>
   <si>
-    <t>combustivel</t>
+    <t>combustível</t>
   </si>
   <si>
     <t>Opcional. gasoline, ethanol, diesel, cng, electric.</t>
   </si>
   <si>
-    <t>A placa precisa existir na aba veiculos ou no banco.</t>
+    <t>A placa precisa existir na aba veículos ou no banco.</t>
   </si>
   <si>
     <t>Se informar CNH, ela precisa existir na aba motoristas ou no banco.</t>
@@ -286,10 +286,10 @@
     <t>Por padrao, litros x preco_litro precisa bater com valor_total. Na tela ha opcao para recalcular valor_total automaticamente.</t>
   </si>
   <si>
-    <t>Para km/l por abastecimento, informe odometro em abastecimentos consecutivos do mesmo veiculo.</t>
-  </si>
-  <si>
-    <t>manutencoes</t>
+    <t>Para km/l por abastecimento, informe odômetro em abastecimentos consecutivos do mesmo veículo.</t>
+  </si>
+  <si>
+    <t>manutenções</t>
   </si>
   <si>
     <t>Opcional. preventive, corrective, predictive.</t>
@@ -307,7 +307,7 @@
     <t>agendamento</t>
   </si>
   <si>
-    <t>Opcional. Km da manutencao.</t>
+    <t>Opcional. Km da manutenção.</t>
   </si>
   <si>
     <t>valor_total</t>
@@ -319,13 +319,13 @@
     <t>descricao</t>
   </si>
   <si>
-    <t>Opcional. Descricao do servico.</t>
-  </si>
-  <si>
-    <t>Se valor_total ficar vazio, sera gravado como zero.</t>
-  </si>
-  <si>
-    <t>Manutencoes entram nos custos acumulados da dashboard.</t>
+    <t>Opcional. Descricao do serviço.</t>
+  </si>
+  <si>
+    <t>Se valor_total ficar vazio, será gravado como zero.</t>
+  </si>
+  <si>
+    <t>Manutenções entram nos custos acumulados da dashboard.</t>
   </si>
   <si>
     <t>documentos</t>
@@ -340,7 +340,7 @@
     <t>referencia *</t>
   </si>
   <si>
-    <t>Obrigatorio. Placa do veiculo ou CNH do motorista.</t>
+    <t>Obrigatorio. Placa do veículo ou CNH do motorista.</t>
   </si>
   <si>
     <t>documento *</t>
@@ -367,7 +367,7 @@
     <t>Opcional. URL publica do arquivo.</t>
   </si>
   <si>
-    <t>entidade aceita vehicle/driver ou veiculo/motorista.</t>
+    <t>entidade aceita vehicle/driver ou veículo/motorista.</t>
   </si>
   <si>
     <t>referencia precisa existir: placa para vehicle, CNH para driver.</t>
@@ -394,7 +394,7 @@
     <t>available</t>
   </si>
   <si>
-    <t>Operacao</t>
+    <t>Operação</t>
   </si>
   <si>
     <t>Logistica</t>

</xml_diff>